<commit_message>
One more year of data.
</commit_message>
<xml_diff>
--- a/drugs/medicine.xlsx
+++ b/drugs/medicine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\lucent\health-data\drugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E623D956-4AAC-4998-B84B-DBFF8BA44F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0CCFA89-F2B1-465A-8D9B-23775E24F6DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1800" windowWidth="28140" windowHeight="19425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8010" yWindow="870" windowWidth="30375" windowHeight="20505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="51">
   <si>
     <t>Date</t>
   </si>
@@ -55,19 +55,149 @@
   </si>
   <si>
     <t>Lot</t>
+  </si>
+  <si>
+    <t>R R Stomach</t>
+  </si>
+  <si>
+    <t>Expiry</t>
+  </si>
+  <si>
+    <t>D735992D</t>
+  </si>
+  <si>
+    <t>Subjective strength</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>very low</t>
+  </si>
+  <si>
+    <t>Serial</t>
+  </si>
+  <si>
+    <t>D746439A</t>
+  </si>
+  <si>
+    <t>369574751668</t>
+  </si>
+  <si>
+    <t>309736030503</t>
+  </si>
+  <si>
+    <t>R T Stomach</t>
+  </si>
+  <si>
+    <t>L L Stomach</t>
+  </si>
+  <si>
+    <t>L T Stomach</t>
+  </si>
+  <si>
+    <t>very high</t>
+  </si>
+  <si>
+    <t>R L Stomach</t>
+  </si>
+  <si>
+    <t>D736216D</t>
+  </si>
+  <si>
+    <t>313084754648</t>
+  </si>
+  <si>
+    <t>D738490D</t>
+  </si>
+  <si>
+    <t>323563906677</t>
+  </si>
+  <si>
+    <t>L UU Stomach</t>
+  </si>
+  <si>
+    <t>L Thigh</t>
+  </si>
+  <si>
+    <t>delayed onset</t>
+  </si>
+  <si>
+    <t>349319171777</t>
+  </si>
+  <si>
+    <t>D790193A</t>
+  </si>
+  <si>
+    <t>321179678092</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>D772233C</t>
+  </si>
+  <si>
+    <t>388462861905</t>
+  </si>
+  <si>
+    <t>D793672D</t>
+  </si>
+  <si>
+    <t>096594151986</t>
+  </si>
+  <si>
+    <t>metformin XR 500</t>
+  </si>
+  <si>
+    <t>high start low end</t>
+  </si>
+  <si>
+    <t>D814653D</t>
+  </si>
+  <si>
+    <t>388082724768</t>
+  </si>
+  <si>
+    <t>095399808123</t>
+  </si>
+  <si>
+    <t>M Stomach</t>
+  </si>
+  <si>
+    <t>D863001A</t>
+  </si>
+  <si>
+    <t>351794997754</t>
+  </si>
+  <si>
+    <t>D837896D</t>
+  </si>
+  <si>
+    <t>383877302654</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -93,9 +223,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -376,15 +508,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -400,8 +537,17 @@
       <c r="E1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>45552.541666666664</v>
       </c>
@@ -414,8 +560,20 @@
       <c r="D2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="3">
+        <v>46102</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>45559.5</v>
       </c>
@@ -428,8 +586,20 @@
       <c r="D3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3">
+        <v>46102</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>45566.5</v>
       </c>
@@ -442,8 +612,20 @@
       <c r="D4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="3">
+        <v>46102</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>45573.5</v>
       </c>
@@ -456,8 +638,1114 @@
       <c r="D5" t="s">
         <v>8</v>
       </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="3">
+        <v>46102</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>45580.5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="3">
+        <v>46141</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45587.5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3">
+        <v>46141</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>45594.583333333336</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="3">
+        <v>46141</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>45601.5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="3">
+        <v>46141</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>45608.5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="3">
+        <v>46139</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>45615.5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="3">
+        <v>46139</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>45622.5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="3">
+        <v>46139</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>45629.5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13">
+        <v>5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="3">
+        <v>46139</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>45636.75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>45645.5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>45650.583333333336</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>45657.5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>45664.541666666664</v>
+      </c>
+      <c r="B18" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18">
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>45671.625</v>
+      </c>
+      <c r="B19" t="s">
+        <v>2</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>45678.645833333336</v>
+      </c>
+      <c r="B20" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>45685.541666666664</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="3">
+        <v>46154</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>45692.604166666664</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" s="3">
+        <v>46178</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>45699.5625</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>5</v>
+      </c>
+      <c r="E23" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" s="3">
+        <v>46178</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H23" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>45706.625</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="3">
+        <v>46178</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>45713.625</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25">
+        <v>5</v>
+      </c>
+      <c r="D25" t="s">
+        <v>5</v>
+      </c>
+      <c r="E25" t="s">
+        <v>34</v>
+      </c>
+      <c r="F25" s="3">
+        <v>46178</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>45720.583333333336</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2</v>
+      </c>
+      <c r="C26">
+        <v>7.5</v>
+      </c>
+      <c r="D26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" s="3">
+        <v>46258</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H26" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>45727.645833333336</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27">
+        <v>7.5</v>
+      </c>
+      <c r="D27" t="s">
+        <v>5</v>
+      </c>
+      <c r="E27" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" s="3">
+        <v>46258</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H27" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>45734.645833333336</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2</v>
+      </c>
+      <c r="C28">
+        <v>7.5</v>
+      </c>
+      <c r="D28" t="s">
+        <v>6</v>
+      </c>
+      <c r="E28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" s="3">
+        <v>46258</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H28" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>45741.583333333336</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C29">
+        <v>7.5</v>
+      </c>
+      <c r="D29" t="s">
+        <v>5</v>
+      </c>
+      <c r="E29" t="s">
+        <v>37</v>
+      </c>
+      <c r="F29" s="3">
+        <v>46258</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H29" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>45748.666666666664</v>
+      </c>
+      <c r="B30" t="s">
+        <v>2</v>
+      </c>
+      <c r="C30">
+        <v>7.5</v>
+      </c>
+      <c r="D30" t="s">
+        <v>6</v>
+      </c>
+      <c r="E30" t="s">
+        <v>39</v>
+      </c>
+      <c r="F30" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H30" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>45755.8125</v>
+      </c>
+      <c r="B31" t="s">
+        <v>2</v>
+      </c>
+      <c r="C31">
+        <v>7.5</v>
+      </c>
+      <c r="D31" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" t="s">
+        <v>39</v>
+      </c>
+      <c r="F31" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H31" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>45762.645833333336</v>
+      </c>
+      <c r="B32" t="s">
+        <v>2</v>
+      </c>
+      <c r="C32">
+        <v>7.5</v>
+      </c>
+      <c r="D32" t="s">
+        <v>6</v>
+      </c>
+      <c r="E32" t="s">
+        <v>39</v>
+      </c>
+      <c r="F32" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H32" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>45769.666666666664</v>
+      </c>
+      <c r="B33" t="s">
+        <v>2</v>
+      </c>
+      <c r="C33">
+        <v>7.5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>5</v>
+      </c>
+      <c r="E33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F33" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H33" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>45776.666666666664</v>
+      </c>
+      <c r="B34" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34">
+        <v>7.5</v>
+      </c>
+      <c r="D34" t="s">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>39</v>
+      </c>
+      <c r="F34" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H34" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>45783.708333333336</v>
+      </c>
+      <c r="B35" t="s">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>7.5</v>
+      </c>
+      <c r="D35" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" t="s">
+        <v>39</v>
+      </c>
+      <c r="F35" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>45790.666666666664</v>
+      </c>
+      <c r="B36" t="s">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>7.5</v>
+      </c>
+      <c r="D36" t="s">
+        <v>6</v>
+      </c>
+      <c r="E36" t="s">
+        <v>39</v>
+      </c>
+      <c r="F36" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>45797.624999884261</v>
+      </c>
+      <c r="B37" t="s">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>7.5</v>
+      </c>
+      <c r="D37" t="s">
+        <v>5</v>
+      </c>
+      <c r="E37" t="s">
+        <v>39</v>
+      </c>
+      <c r="F37" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>45804.666666666664</v>
+      </c>
+      <c r="B38" t="s">
+        <v>2</v>
+      </c>
+      <c r="C38">
+        <v>10</v>
+      </c>
+      <c r="D38" t="s">
+        <v>6</v>
+      </c>
+      <c r="E38" t="s">
+        <v>43</v>
+      </c>
+      <c r="F38" s="3">
+        <v>46385</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>45811.625</v>
+      </c>
+      <c r="B39" t="s">
+        <v>2</v>
+      </c>
+      <c r="C39">
+        <v>10</v>
+      </c>
+      <c r="D39" t="s">
+        <v>5</v>
+      </c>
+      <c r="E39" t="s">
+        <v>43</v>
+      </c>
+      <c r="F39" s="3">
+        <v>46385</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>45818.625</v>
+      </c>
+      <c r="B40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C40">
+        <v>10</v>
+      </c>
+      <c r="D40" t="s">
+        <v>6</v>
+      </c>
+      <c r="E40" t="s">
+        <v>43</v>
+      </c>
+      <c r="F40" s="3">
+        <v>46385</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>45825.666666666664</v>
+      </c>
+      <c r="B41" t="s">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>10</v>
+      </c>
+      <c r="D41" t="s">
+        <v>5</v>
+      </c>
+      <c r="E41" t="s">
+        <v>43</v>
+      </c>
+      <c r="F41" s="3">
+        <v>46385</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>45832.70833321759</v>
+      </c>
+      <c r="B42" t="s">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>10</v>
+      </c>
+      <c r="D42" t="s">
+        <v>6</v>
+      </c>
+      <c r="E42" t="s">
+        <v>47</v>
+      </c>
+      <c r="F42" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>45839.666666666664</v>
+      </c>
+      <c r="B43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>10</v>
+      </c>
+      <c r="D43" t="s">
+        <v>5</v>
+      </c>
+      <c r="E43" t="s">
+        <v>47</v>
+      </c>
+      <c r="F43" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>45846.708333333336</v>
+      </c>
+      <c r="B44" t="s">
+        <v>2</v>
+      </c>
+      <c r="C44">
+        <v>10</v>
+      </c>
+      <c r="D44" t="s">
+        <v>6</v>
+      </c>
+      <c r="E44" t="s">
+        <v>47</v>
+      </c>
+      <c r="F44" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>45853.999305555553</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>10</v>
+      </c>
+      <c r="D45" t="s">
+        <v>46</v>
+      </c>
+      <c r="E45" t="s">
+        <v>47</v>
+      </c>
+      <c r="F45" s="3">
+        <v>46317</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>45860.708333333336</v>
+      </c>
+      <c r="B46" t="s">
+        <v>2</v>
+      </c>
+      <c r="C46">
+        <v>10</v>
+      </c>
+      <c r="D46" t="s">
+        <v>5</v>
+      </c>
+      <c r="E46" t="s">
+        <v>49</v>
+      </c>
+      <c r="F46" s="3">
+        <v>46457</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>45867.8125</v>
+      </c>
+      <c r="B47" t="s">
+        <v>2</v>
+      </c>
+      <c r="C47">
+        <v>10</v>
+      </c>
+      <c r="D47" t="s">
+        <v>6</v>
+      </c>
+      <c r="E47" t="s">
+        <v>49</v>
+      </c>
+      <c r="F47" s="3">
+        <v>46457</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>45874.770833333336</v>
+      </c>
+      <c r="B48" t="s">
+        <v>2</v>
+      </c>
+      <c r="C48">
+        <v>10</v>
+      </c>
+      <c r="D48" t="s">
+        <v>5</v>
+      </c>
+      <c r="E48" t="s">
+        <v>49</v>
+      </c>
+      <c r="F48" s="3">
+        <v>46457</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>45881.708333333336</v>
+      </c>
+      <c r="B49" t="s">
+        <v>2</v>
+      </c>
+      <c r="C49">
+        <v>10</v>
+      </c>
+      <c r="D49" t="s">
+        <v>6</v>
+      </c>
+      <c r="E49" t="s">
+        <v>49</v>
+      </c>
+      <c r="F49" s="3">
+        <v>46457</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>45747.5</v>
+      </c>
+      <c r="B50" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>45748.5</v>
+      </c>
+      <c r="B51" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>45748.875</v>
+      </c>
+      <c r="B52" t="s">
+        <v>41</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
2 more months of intake, weight, workouts
</commit_message>
<xml_diff>
--- a/drugs/medicine.xlsx
+++ b/drugs/medicine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\lucent\health-data\drugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0CCFA89-F2B1-465A-8D9B-23775E24F6DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B797610F-C850-406D-9A4F-D65A5C8017E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8010" yWindow="870" windowWidth="30375" windowHeight="20505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7875" yWindow="3885" windowWidth="21345" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="56">
   <si>
     <t>Date</t>
   </si>
@@ -178,6 +178,21 @@
   </si>
   <si>
     <t>383877302654</t>
+  </si>
+  <si>
+    <t>D886383C</t>
+  </si>
+  <si>
+    <t>309165048682</t>
+  </si>
+  <si>
+    <t>D886927</t>
+  </si>
+  <si>
+    <t>336281748568</t>
+  </si>
+  <si>
+    <t>353095929440</t>
   </si>
 </sst>
 </file>
@@ -508,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1699,7 +1714,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>45881.708333333336</v>
+        <v>45881.791666666664</v>
       </c>
       <c r="B49" t="s">
         <v>2</v>
@@ -1722,25 +1737,301 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>45747.5</v>
+        <v>45888.729166666664</v>
       </c>
       <c r="B50" t="s">
-        <v>41</v>
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>12.5</v>
+      </c>
+      <c r="D50" t="s">
+        <v>5</v>
+      </c>
+      <c r="E50" t="s">
+        <v>51</v>
+      </c>
+      <c r="F50" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>45748.5</v>
+        <v>45895.75</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>2</v>
+      </c>
+      <c r="C51">
+        <v>12.5</v>
+      </c>
+      <c r="D51" t="s">
+        <v>6</v>
+      </c>
+      <c r="E51" t="s">
+        <v>51</v>
+      </c>
+      <c r="F51" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
+        <v>45902.770833333336</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2</v>
+      </c>
+      <c r="C52">
+        <v>12.5</v>
+      </c>
+      <c r="D52" t="s">
+        <v>5</v>
+      </c>
+      <c r="E52" t="s">
+        <v>51</v>
+      </c>
+      <c r="F52" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>45909.791666666664</v>
+      </c>
+      <c r="B53" t="s">
+        <v>2</v>
+      </c>
+      <c r="C53">
+        <v>12.5</v>
+      </c>
+      <c r="D53" t="s">
+        <v>6</v>
+      </c>
+      <c r="E53" t="s">
+        <v>51</v>
+      </c>
+      <c r="F53" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>45916.791666666664</v>
+      </c>
+      <c r="B54" t="s">
+        <v>2</v>
+      </c>
+      <c r="C54">
+        <v>12.5</v>
+      </c>
+      <c r="D54" t="s">
+        <v>5</v>
+      </c>
+      <c r="E54" t="s">
+        <v>53</v>
+      </c>
+      <c r="F54" s="3">
+        <v>46516</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>45923.791666608799</v>
+      </c>
+      <c r="B55" t="s">
+        <v>2</v>
+      </c>
+      <c r="C55">
+        <v>12.5</v>
+      </c>
+      <c r="D55" t="s">
+        <v>6</v>
+      </c>
+      <c r="E55" t="s">
+        <v>53</v>
+      </c>
+      <c r="F55" s="3">
+        <v>46516</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>45930.770833333336</v>
+      </c>
+      <c r="B56" t="s">
+        <v>2</v>
+      </c>
+      <c r="C56">
+        <v>12.5</v>
+      </c>
+      <c r="D56" t="s">
+        <v>5</v>
+      </c>
+      <c r="E56" t="s">
+        <v>53</v>
+      </c>
+      <c r="F56" s="3">
+        <v>46516</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>45937.791666608799</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2</v>
+      </c>
+      <c r="C57">
+        <v>12.5</v>
+      </c>
+      <c r="D57" t="s">
+        <v>6</v>
+      </c>
+      <c r="E57" t="s">
+        <v>53</v>
+      </c>
+      <c r="F57" s="3">
+        <v>46516</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>45944.791666666664</v>
+      </c>
+      <c r="B58" t="s">
+        <v>2</v>
+      </c>
+      <c r="C58">
+        <v>12.5</v>
+      </c>
+      <c r="D58" t="s">
+        <v>5</v>
+      </c>
+      <c r="E58" t="s">
+        <v>51</v>
+      </c>
+      <c r="F58" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>45951.854166666664</v>
+      </c>
+      <c r="B59" t="s">
+        <v>2</v>
+      </c>
+      <c r="C59">
+        <v>12.5</v>
+      </c>
+      <c r="D59" t="s">
+        <v>6</v>
+      </c>
+      <c r="E59" t="s">
+        <v>51</v>
+      </c>
+      <c r="F59" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>45958.791666666664</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2</v>
+      </c>
+      <c r="C60">
+        <v>12.5</v>
+      </c>
+      <c r="D60" t="s">
+        <v>5</v>
+      </c>
+      <c r="E60" t="s">
+        <v>51</v>
+      </c>
+      <c r="F60" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>45965.87499971065</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2</v>
+      </c>
+      <c r="C61">
+        <v>12.5</v>
+      </c>
+      <c r="D61" t="s">
+        <v>6</v>
+      </c>
+      <c r="E61" t="s">
+        <v>51</v>
+      </c>
+      <c r="F61" s="3">
+        <v>46513</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>45747.5</v>
+      </c>
+      <c r="B62" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>45748.5</v>
+      </c>
+      <c r="B63" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
         <v>45748.875</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B64" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild extraction pipeline. Add 2+ years of data. Remove old parsers
  - Replace Go/JS/Python intake parsers with idempotent HTML+OXPS extractors and merge.py
  - Add intake verification, sanity check, and cross-extractor comparison scripts
  - Steps/sleep extractor now pulls directly from Samsung Health 7z backups (no raw CSVs in repo)
  - Add temperature, fatty acids, trips, weight extraction, and sleep/steps CSVs
</commit_message>
<xml_diff>
--- a/drugs/medicine.xlsx
+++ b/drugs/medicine.xlsx
@@ -1,31 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\lucent\health-data\drugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B797610F-C850-406D-9A4F-D65A5C8017E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78EF198F-B7D8-4318-ACF3-82932C9BFE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7875" yWindow="3885" windowWidth="21345" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="80">
   <si>
     <t>Date</t>
   </si>
@@ -33,75 +28,75 @@
     <t>Drug</t>
   </si>
   <si>
+    <t>Dose (mg)</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Lot</t>
+  </si>
+  <si>
+    <t>Expiry</t>
+  </si>
+  <si>
+    <t>Serial</t>
+  </si>
+  <si>
+    <t>Subjective strength</t>
+  </si>
+  <si>
     <t>Zepbound (tirzepatide)</t>
   </si>
   <si>
-    <t>Location</t>
-  </si>
-  <si>
     <t>R Thigh</t>
   </si>
   <si>
+    <t>D746439A</t>
+  </si>
+  <si>
+    <t>369574751668</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
     <t>L Stomach</t>
   </si>
   <si>
+    <t>high</t>
+  </si>
+  <si>
     <t>R Stomach</t>
   </si>
   <si>
-    <t>Dose (mg)</t>
-  </si>
-  <si>
     <t>B Stomach</t>
   </si>
   <si>
-    <t>Lot</t>
+    <t>very low</t>
   </si>
   <si>
     <t>R R Stomach</t>
   </si>
   <si>
-    <t>Expiry</t>
-  </si>
-  <si>
     <t>D735992D</t>
   </si>
   <si>
-    <t>Subjective strength</t>
-  </si>
-  <si>
-    <t>low</t>
-  </si>
-  <si>
-    <t>high</t>
-  </si>
-  <si>
-    <t>very low</t>
-  </si>
-  <si>
-    <t>Serial</t>
-  </si>
-  <si>
-    <t>D746439A</t>
-  </si>
-  <si>
-    <t>369574751668</t>
-  </si>
-  <si>
     <t>309736030503</t>
   </si>
   <si>
+    <t>very high</t>
+  </si>
+  <si>
+    <t>L L Stomach</t>
+  </si>
+  <si>
     <t>R T Stomach</t>
   </si>
   <si>
-    <t>L L Stomach</t>
-  </si>
-  <si>
     <t>L T Stomach</t>
   </si>
   <si>
-    <t>very high</t>
-  </si>
-  <si>
     <t>R L Stomach</t>
   </si>
   <si>
@@ -111,15 +106,15 @@
     <t>313084754648</t>
   </si>
   <si>
+    <t>L UU Stomach</t>
+  </si>
+  <si>
     <t>D738490D</t>
   </si>
   <si>
     <t>323563906677</t>
   </si>
   <si>
-    <t>L UU Stomach</t>
-  </si>
-  <si>
     <t>L Thigh</t>
   </si>
   <si>
@@ -150,69 +145,136 @@
     <t>096594151986</t>
   </si>
   <si>
+    <t>high start low end</t>
+  </si>
+  <si>
+    <t>095399808123</t>
+  </si>
+  <si>
+    <t>D814653D</t>
+  </si>
+  <si>
+    <t>388082724768</t>
+  </si>
+  <si>
+    <t>D863001A</t>
+  </si>
+  <si>
+    <t>351794997754</t>
+  </si>
+  <si>
+    <t>M Stomach</t>
+  </si>
+  <si>
+    <t>D837896D</t>
+  </si>
+  <si>
+    <t>383877302654</t>
+  </si>
+  <si>
+    <t>D886383C</t>
+  </si>
+  <si>
+    <t>309165048682</t>
+  </si>
+  <si>
+    <t>D886927</t>
+  </si>
+  <si>
+    <t>336281748568</t>
+  </si>
+  <si>
+    <t>353095929440</t>
+  </si>
+  <si>
+    <t>D881140C</t>
+  </si>
+  <si>
+    <t>390595030960</t>
+  </si>
+  <si>
+    <t>D871561E</t>
+  </si>
+  <si>
+    <t>342402864610</t>
+  </si>
+  <si>
+    <t>D886290J</t>
+  </si>
+  <si>
+    <t>392811739144</t>
+  </si>
+  <si>
     <t>metformin XR 500</t>
   </si>
   <si>
-    <t>high start low end</t>
-  </si>
-  <si>
-    <t>D814653D</t>
-  </si>
-  <si>
-    <t>388082724768</t>
-  </si>
-  <si>
-    <t>095399808123</t>
-  </si>
-  <si>
-    <t>M Stomach</t>
-  </si>
-  <si>
-    <t>D863001A</t>
-  </si>
-  <si>
-    <t>351794997754</t>
-  </si>
-  <si>
-    <t>D837896D</t>
-  </si>
-  <si>
-    <t>383877302654</t>
-  </si>
-  <si>
-    <t>D886383C</t>
-  </si>
-  <si>
-    <t>309165048682</t>
-  </si>
-  <si>
-    <t>D886927</t>
-  </si>
-  <si>
-    <t>336281748568</t>
-  </si>
-  <si>
-    <t>353095929440</t>
+    <t>Pfizer BioNTech COVID-19 vaccine</t>
+  </si>
+  <si>
+    <t>ETCH</t>
+  </si>
+  <si>
+    <t>EK5730</t>
+  </si>
+  <si>
+    <t>EL0142</t>
+  </si>
+  <si>
+    <t>Kroger 848</t>
+  </si>
+  <si>
+    <t>FE3592</t>
+  </si>
+  <si>
+    <t>Moderna COVID-19 Bivalent vaccine</t>
+  </si>
+  <si>
+    <t>CVS 04624</t>
+  </si>
+  <si>
+    <t>AS7144B</t>
+  </si>
+  <si>
+    <t>Moderna 2023-24 COVID-19 vaccine</t>
+  </si>
+  <si>
+    <t>CVS 06363</t>
+  </si>
+  <si>
+    <t>3030368</t>
+  </si>
+  <si>
+    <t>Pfizer 2024-25 COVID-19 vaccine</t>
+  </si>
+  <si>
+    <t>CVS 11137</t>
+  </si>
+  <si>
+    <t>LM2223</t>
+  </si>
+  <si>
+    <t>D931135G</t>
+  </si>
+  <si>
+    <t>322366636070</t>
+  </si>
+  <si>
+    <t>389001989216</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -238,11 +300,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,20 +586,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H64"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H95"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -544,143 +607,143 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>45552.541666666664</v>
+        <v>45552.541666666657</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C2">
         <v>2.5</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F2" s="3">
         <v>46102</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>45559.5</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>2.5</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F3" s="3">
         <v>46102</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>45566.5</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>2.5</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F4" s="3">
         <v>46102</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>45573.5</v>
       </c>
       <c r="B5" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>2.5</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F5" s="3">
         <v>46102</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>45580.5</v>
       </c>
       <c r="B6" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F6" s="3">
         <v>46141</v>
@@ -689,15 +752,15 @@
         <v>20</v>
       </c>
       <c r="H6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>45587.5</v>
       </c>
       <c r="B7" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -706,7 +769,7 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F7" s="3">
         <v>46141</v>
@@ -715,24 +778,24 @@
         <v>20</v>
       </c>
       <c r="H7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
-        <v>45594.583333333336</v>
+        <v>45594.583333333343</v>
       </c>
       <c r="B8" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C8">
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F8" s="3">
         <v>46141</v>
@@ -741,24 +804,24 @@
         <v>20</v>
       </c>
       <c r="H8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>45601.5</v>
       </c>
       <c r="B9" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C9">
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F9" s="3">
         <v>46141</v>
@@ -767,15 +830,15 @@
         <v>20</v>
       </c>
       <c r="H9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>45608.5</v>
       </c>
       <c r="B10" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C10">
         <v>5</v>
@@ -793,12 +856,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>45615.5</v>
       </c>
       <c r="B11" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C11">
         <v>5</v>
@@ -813,12 +876,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>45622.5</v>
       </c>
       <c r="B12" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C12">
         <v>5</v>
@@ -833,12 +896,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>45629.5</v>
       </c>
       <c r="B13" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C13">
         <v>5</v>
@@ -853,35 +916,35 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>45636.75</v>
       </c>
       <c r="B14" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C14">
         <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F14" s="3">
         <v>46154</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>45645.5</v>
       </c>
       <c r="B15" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C15">
         <v>5</v>
@@ -890,85 +953,85 @@
         <v>31</v>
       </c>
       <c r="E15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F15" s="3">
         <v>46154</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
-        <v>45650.583333333336</v>
+        <v>45650.583333333343</v>
       </c>
       <c r="B16" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C16">
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F16" s="3">
         <v>46154</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>45657.5</v>
       </c>
       <c r="B17" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C17">
         <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F17" s="3">
         <v>46154</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
-        <v>45664.541666666664</v>
+        <v>45664.541666666657</v>
       </c>
       <c r="B18" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C18">
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F18" s="3">
         <v>46154</v>
@@ -977,24 +1040,24 @@
         <v>33</v>
       </c>
       <c r="H18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>45671.625</v>
       </c>
       <c r="B19" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C19">
         <v>5</v>
       </c>
       <c r="D19" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F19" s="3">
         <v>46154</v>
@@ -1003,24 +1066,24 @@
         <v>33</v>
       </c>
       <c r="H19" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>45678.645833333336</v>
+        <v>45678.645833333343</v>
       </c>
       <c r="B20" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C20">
         <v>5</v>
       </c>
       <c r="D20" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F20" s="3">
         <v>46154</v>
@@ -1029,21 +1092,21 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>45685.541666666664</v>
+        <v>45685.541666666657</v>
       </c>
       <c r="B21" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F21" s="3">
         <v>46154</v>
@@ -1052,18 +1115,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
-        <v>45692.604166666664</v>
+        <v>45692.604166666657</v>
       </c>
       <c r="B22" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C22">
         <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E22" t="s">
         <v>34</v>
@@ -1075,18 +1138,18 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>45699.5625</v>
       </c>
       <c r="B23" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C23">
         <v>5</v>
       </c>
       <c r="D23" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E23" t="s">
         <v>34</v>
@@ -1098,21 +1161,21 @@
         <v>35</v>
       </c>
       <c r="H23" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>45706.625</v>
       </c>
       <c r="B24" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C24">
         <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E24" t="s">
         <v>34</v>
@@ -1127,18 +1190,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>45713.625</v>
       </c>
       <c r="B25" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C25">
         <v>5</v>
       </c>
       <c r="D25" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E25" t="s">
         <v>34</v>
@@ -1150,21 +1213,21 @@
         <v>35</v>
       </c>
       <c r="H25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
-        <v>45720.583333333336</v>
+        <v>45720.583333333343</v>
       </c>
       <c r="B26" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C26">
         <v>7.5</v>
       </c>
       <c r="D26" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E26" t="s">
         <v>37</v>
@@ -1179,18 +1242,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>45727.645833333336</v>
+        <v>45727.645833333343</v>
       </c>
       <c r="B27" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C27">
         <v>7.5</v>
       </c>
       <c r="D27" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E27" t="s">
         <v>37</v>
@@ -1205,18 +1268,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>45734.645833333336</v>
+        <v>45734.645833333343</v>
       </c>
       <c r="B28" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C28">
         <v>7.5</v>
       </c>
       <c r="D28" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E28" t="s">
         <v>37</v>
@@ -1228,21 +1291,21 @@
         <v>38</v>
       </c>
       <c r="H28" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>45741.583333333336</v>
+        <v>45741.583333333343</v>
       </c>
       <c r="B29" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C29">
         <v>7.5</v>
       </c>
       <c r="D29" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E29" t="s">
         <v>37</v>
@@ -1257,18 +1320,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>45748.666666666664</v>
+        <v>45748.666666666657</v>
       </c>
       <c r="B30" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C30">
         <v>7.5</v>
       </c>
       <c r="D30" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E30" t="s">
         <v>39</v>
@@ -1283,18 +1346,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>45755.8125</v>
       </c>
       <c r="B31" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C31">
         <v>7.5</v>
       </c>
       <c r="D31" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
         <v>39</v>
@@ -1306,21 +1369,21 @@
         <v>40</v>
       </c>
       <c r="H31" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
-        <v>45762.645833333336</v>
+        <v>45762.645833333343</v>
       </c>
       <c r="B32" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C32">
         <v>7.5</v>
       </c>
       <c r="D32" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E32" t="s">
         <v>39</v>
@@ -1332,21 +1395,21 @@
         <v>40</v>
       </c>
       <c r="H32" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>45769.666666666664</v>
+        <v>45769.666666666657</v>
       </c>
       <c r="B33" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C33">
         <v>7.5</v>
       </c>
       <c r="D33" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E33" t="s">
         <v>39</v>
@@ -1358,21 +1421,21 @@
         <v>40</v>
       </c>
       <c r="H33" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
-        <v>45776.666666666664</v>
+        <v>45776.666666666657</v>
       </c>
       <c r="B34" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C34">
         <v>7.5</v>
       </c>
       <c r="D34" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E34" t="s">
         <v>39</v>
@@ -1381,24 +1444,24 @@
         <v>46317</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H34" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
-        <v>45783.708333333336</v>
+        <v>45783.708333333343</v>
       </c>
       <c r="B35" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C35">
         <v>7.5</v>
       </c>
       <c r="D35" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
         <v>39</v>
@@ -1407,24 +1470,24 @@
         <v>46317</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H35" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
-        <v>45790.666666666664</v>
+        <v>45790.666666666657</v>
       </c>
       <c r="B36" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C36">
         <v>7.5</v>
       </c>
       <c r="D36" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E36" t="s">
         <v>39</v>
@@ -1433,21 +1496,21 @@
         <v>46317</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>45797.624999884261</v>
       </c>
       <c r="B37" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C37">
         <v>7.5</v>
       </c>
       <c r="D37" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E37" t="s">
         <v>39</v>
@@ -1456,21 +1519,21 @@
         <v>46317</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
-        <v>45804.666666666664</v>
+        <v>45804.666666666657</v>
       </c>
       <c r="B38" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E38" t="s">
         <v>43</v>
@@ -1482,18 +1545,18 @@
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>45811.625</v>
       </c>
       <c r="B39" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C39">
         <v>10</v>
       </c>
       <c r="D39" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s">
         <v>43</v>
@@ -1505,18 +1568,18 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>45818.625</v>
       </c>
       <c r="B40" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C40">
         <v>10</v>
       </c>
       <c r="D40" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E40" t="s">
         <v>43</v>
@@ -1528,18 +1591,18 @@
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
-        <v>45825.666666666664</v>
+        <v>45825.666666666657</v>
       </c>
       <c r="B41" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C41">
         <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E41" t="s">
         <v>43</v>
@@ -1551,492 +1614,1035 @@
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>45832.70833321759</v>
       </c>
       <c r="B42" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C42">
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E42" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F42" s="3">
         <v>46317</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
-        <v>45839.666666666664</v>
+        <v>45839.666666666657</v>
       </c>
       <c r="B43" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C43">
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E43" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F43" s="3">
         <v>46317</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
-        <v>45846.708333333336</v>
+        <v>45846.708333333343</v>
       </c>
       <c r="B44" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C44">
         <v>10</v>
       </c>
       <c r="D44" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E44" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F44" s="3">
         <v>46317</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>45853.999305555553</v>
       </c>
       <c r="B45" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C45">
         <v>10</v>
       </c>
       <c r="D45" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E45" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F45" s="3">
         <v>46317</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
-        <v>45860.708333333336</v>
+        <v>45860.708333333343</v>
       </c>
       <c r="B46" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C46">
         <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F46" s="3">
         <v>46457</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>45867.8125</v>
       </c>
       <c r="B47" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C47">
         <v>10</v>
       </c>
       <c r="D47" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F47" s="3">
         <v>46457</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
-        <v>45874.770833333336</v>
+        <v>45874.770833333343</v>
       </c>
       <c r="B48" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C48">
         <v>10</v>
       </c>
       <c r="D48" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F48" s="3">
         <v>46457</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
-        <v>45881.791666666664</v>
+        <v>45881.791666666657</v>
       </c>
       <c r="B49" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C49">
         <v>10</v>
       </c>
       <c r="D49" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F49" s="3">
         <v>46457</v>
       </c>
       <c r="G49" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>45888.729166666657</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50">
+        <v>12.5</v>
+      </c>
+      <c r="D50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
-        <v>45888.729166666664</v>
-      </c>
-      <c r="B50" t="s">
-        <v>2</v>
-      </c>
-      <c r="C50">
-        <v>12.5</v>
-      </c>
-      <c r="D50" t="s">
-        <v>5</v>
-      </c>
-      <c r="E50" t="s">
-        <v>51</v>
       </c>
       <c r="F50" s="3">
         <v>46513</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>45895.75</v>
       </c>
       <c r="B51" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C51">
         <v>12.5</v>
       </c>
       <c r="D51" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F51" s="3">
         <v>46513</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
-        <v>45902.770833333336</v>
+        <v>45902.770833333343</v>
       </c>
       <c r="B52" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C52">
         <v>12.5</v>
       </c>
       <c r="D52" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E52" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F52" s="3">
         <v>46513</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
-        <v>45909.791666666664</v>
+        <v>45909.791666666657</v>
       </c>
       <c r="B53" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C53">
         <v>12.5</v>
       </c>
       <c r="D53" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E53" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F53" s="3">
         <v>46513</v>
       </c>
       <c r="G53" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>45916.791666666657</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54">
+        <v>12.5</v>
+      </c>
+      <c r="D54" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="1">
-        <v>45916.791666666664</v>
-      </c>
-      <c r="B54" t="s">
-        <v>2</v>
-      </c>
-      <c r="C54">
-        <v>12.5</v>
-      </c>
-      <c r="D54" t="s">
-        <v>5</v>
-      </c>
-      <c r="E54" t="s">
-        <v>53</v>
       </c>
       <c r="F54" s="3">
         <v>46516</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>45923.791666608799</v>
       </c>
       <c r="B55" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C55">
         <v>12.5</v>
       </c>
       <c r="D55" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E55" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F55" s="3">
         <v>46516</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
-        <v>45930.770833333336</v>
+        <v>45930.770833333343</v>
       </c>
       <c r="B56" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C56">
         <v>12.5</v>
       </c>
       <c r="D56" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E56" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F56" s="3">
         <v>46516</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>45937.791666608799</v>
       </c>
       <c r="B57" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C57">
         <v>12.5</v>
       </c>
       <c r="D57" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E57" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F57" s="3">
         <v>46516</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
-        <v>45944.791666666664</v>
+        <v>45944.791666666657</v>
       </c>
       <c r="B58" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C58">
         <v>12.5</v>
       </c>
       <c r="D58" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E58" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F58" s="3">
         <v>46513</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
-        <v>45951.854166666664</v>
+        <v>45951.854166666657</v>
       </c>
       <c r="B59" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C59">
         <v>12.5</v>
       </c>
       <c r="D59" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E59" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F59" s="3">
         <v>46513</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
-        <v>45958.791666666664</v>
+        <v>45958.791666666657</v>
       </c>
       <c r="B60" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C60">
         <v>12.5</v>
       </c>
       <c r="D60" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E60" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F60" s="3">
         <v>46513</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
-        <v>45965.87499971065</v>
+        <v>45965.75</v>
       </c>
       <c r="B61" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C61">
         <v>12.5</v>
       </c>
       <c r="D61" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E61" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F61" s="3">
         <v>46513</v>
       </c>
       <c r="G61" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>45972.708333391201</v>
+      </c>
+      <c r="B62" t="s">
+        <v>8</v>
+      </c>
+      <c r="C62">
+        <v>12.5</v>
+      </c>
+      <c r="D62" t="s">
+        <v>13</v>
+      </c>
+      <c r="E62" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="1">
+      <c r="F62" s="3">
+        <v>46573</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>45979.75</v>
+      </c>
+      <c r="B63" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63">
+        <v>12.5</v>
+      </c>
+      <c r="D63" t="s">
+        <v>15</v>
+      </c>
+      <c r="E63" t="s">
+        <v>55</v>
+      </c>
+      <c r="F63" s="3">
+        <v>46573</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>45986.8125</v>
+      </c>
+      <c r="B64" t="s">
+        <v>8</v>
+      </c>
+      <c r="C64">
+        <v>12.5</v>
+      </c>
+      <c r="D64" t="s">
+        <v>13</v>
+      </c>
+      <c r="E64" t="s">
+        <v>55</v>
+      </c>
+      <c r="F64" s="3">
+        <v>46573</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>45993.999305555553</v>
+      </c>
+      <c r="B65" t="s">
+        <v>8</v>
+      </c>
+      <c r="C65">
+        <v>12.5</v>
+      </c>
+      <c r="D65" t="s">
+        <v>15</v>
+      </c>
+      <c r="E65" t="s">
+        <v>55</v>
+      </c>
+      <c r="F65" s="3">
+        <v>46573</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
+        <v>46000.916666666657</v>
+      </c>
+      <c r="B66" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66">
+        <v>12.5</v>
+      </c>
+      <c r="D66" t="s">
+        <v>13</v>
+      </c>
+      <c r="E66" t="s">
+        <v>57</v>
+      </c>
+      <c r="F66" s="3">
+        <v>46530</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>46007.75</v>
+      </c>
+      <c r="B67" t="s">
+        <v>8</v>
+      </c>
+      <c r="C67">
+        <v>12.5</v>
+      </c>
+      <c r="D67" t="s">
+        <v>15</v>
+      </c>
+      <c r="E67" t="s">
+        <v>57</v>
+      </c>
+      <c r="F67" s="3">
+        <v>46530</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
+        <v>46014.8125</v>
+      </c>
+      <c r="B68" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68">
+        <v>12.5</v>
+      </c>
+      <c r="D68" t="s">
+        <v>13</v>
+      </c>
+      <c r="E68" t="s">
+        <v>57</v>
+      </c>
+      <c r="F68" s="3">
+        <v>46530</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
+        <v>46021.875</v>
+      </c>
+      <c r="B69" t="s">
+        <v>8</v>
+      </c>
+      <c r="C69">
+        <v>12.5</v>
+      </c>
+      <c r="D69" t="s">
+        <v>15</v>
+      </c>
+      <c r="E69" t="s">
+        <v>57</v>
+      </c>
+      <c r="F69" s="3">
+        <v>46530</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
+        <v>46028.916666666657</v>
+      </c>
+      <c r="B70" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70">
+        <v>12.5</v>
+      </c>
+      <c r="D70" t="s">
+        <v>13</v>
+      </c>
+      <c r="E70" t="s">
+        <v>59</v>
+      </c>
+      <c r="F70" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
+        <v>46035.95833321759</v>
+      </c>
+      <c r="B71" t="s">
+        <v>8</v>
+      </c>
+      <c r="C71">
+        <v>12.5</v>
+      </c>
+      <c r="D71" t="s">
+        <v>15</v>
+      </c>
+      <c r="E71" t="s">
+        <v>59</v>
+      </c>
+      <c r="F71" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" s="1">
+        <v>46042.999305555553</v>
+      </c>
+      <c r="B72" t="s">
+        <v>8</v>
+      </c>
+      <c r="C72">
+        <v>12.5</v>
+      </c>
+      <c r="D72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E72" t="s">
+        <v>59</v>
+      </c>
+      <c r="F72" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" s="1">
+        <v>46049.9375</v>
+      </c>
+      <c r="B73" t="s">
+        <v>8</v>
+      </c>
+      <c r="C73">
+        <v>12.5</v>
+      </c>
+      <c r="D73" t="s">
+        <v>15</v>
+      </c>
+      <c r="E73" t="s">
+        <v>59</v>
+      </c>
+      <c r="F73" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74" s="1">
+        <v>46056.9375</v>
+      </c>
+      <c r="B74" t="s">
+        <v>8</v>
+      </c>
+      <c r="C74">
+        <v>12.5</v>
+      </c>
+      <c r="D74" t="s">
+        <v>13</v>
+      </c>
+      <c r="E74" t="s">
+        <v>59</v>
+      </c>
+      <c r="F74" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
+        <v>46063.998611111107</v>
+      </c>
+      <c r="B75" t="s">
+        <v>8</v>
+      </c>
+      <c r="C75">
+        <v>12.5</v>
+      </c>
+      <c r="D75" t="s">
+        <v>15</v>
+      </c>
+      <c r="E75" t="s">
+        <v>59</v>
+      </c>
+      <c r="F75" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
+        <v>46070.999305555553</v>
+      </c>
+      <c r="B76" t="s">
+        <v>8</v>
+      </c>
+      <c r="C76">
+        <v>12.5</v>
+      </c>
+      <c r="D76" t="s">
+        <v>13</v>
+      </c>
+      <c r="E76" t="s">
+        <v>59</v>
+      </c>
+      <c r="F76" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
+        <v>46077.9375</v>
+      </c>
+      <c r="B77" t="s">
+        <v>8</v>
+      </c>
+      <c r="C77">
+        <v>12.5</v>
+      </c>
+      <c r="D77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E77" t="s">
+        <v>59</v>
+      </c>
+      <c r="F77" s="3">
+        <v>46575</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
+        <v>46084.979166666657</v>
+      </c>
+      <c r="B78" t="s">
+        <v>8</v>
+      </c>
+      <c r="C78">
+        <v>12.5</v>
+      </c>
+      <c r="D78" t="s">
+        <v>13</v>
+      </c>
+      <c r="E78" t="s">
+        <v>77</v>
+      </c>
+      <c r="F78" s="3">
+        <v>46700</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
+        <v>46091.989583333343</v>
+      </c>
+      <c r="B79" t="s">
+        <v>8</v>
+      </c>
+      <c r="C79">
+        <v>12.5</v>
+      </c>
+      <c r="D79" t="s">
+        <v>15</v>
+      </c>
+      <c r="E79" t="s">
+        <v>77</v>
+      </c>
+      <c r="F79" s="3">
+        <v>46700</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
+        <v>46098.999305555553</v>
+      </c>
+      <c r="B80" t="s">
+        <v>8</v>
+      </c>
+      <c r="C80">
+        <v>12.5</v>
+      </c>
+      <c r="D80" t="s">
+        <v>13</v>
+      </c>
+      <c r="E80" t="s">
+        <v>77</v>
+      </c>
+      <c r="F80" s="3">
+        <v>46700</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
+        <v>46105.958333333336</v>
+      </c>
+      <c r="B81" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81">
+        <v>12.5</v>
+      </c>
+      <c r="D81" t="s">
+        <v>15</v>
+      </c>
+      <c r="E81" t="s">
+        <v>77</v>
+      </c>
+      <c r="F81" s="3">
+        <v>46700</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
         <v>45747.5</v>
       </c>
-      <c r="B62" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="1">
+      <c r="B86" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
         <v>45748.5</v>
       </c>
-      <c r="B63" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="1">
+      <c r="B87" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
         <v>45748.875</v>
       </c>
-      <c r="B64" t="s">
-        <v>41</v>
+      <c r="B88" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" s="4">
+        <v>44192.5</v>
+      </c>
+      <c r="B90" t="s">
+        <v>62</v>
+      </c>
+      <c r="D90" t="s">
+        <v>63</v>
+      </c>
+      <c r="E90" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91" s="4">
+        <v>44214.5</v>
+      </c>
+      <c r="B91" t="s">
+        <v>62</v>
+      </c>
+      <c r="D91" t="s">
+        <v>63</v>
+      </c>
+      <c r="E91" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" s="4">
+        <v>44463.5</v>
+      </c>
+      <c r="B92" t="s">
+        <v>62</v>
+      </c>
+      <c r="D92" t="s">
+        <v>66</v>
+      </c>
+      <c r="E92" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A93" s="4">
+        <v>44806.5</v>
+      </c>
+      <c r="B93" t="s">
+        <v>68</v>
+      </c>
+      <c r="D93" t="s">
+        <v>69</v>
+      </c>
+      <c r="E93" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" s="4">
+        <v>45185.5</v>
+      </c>
+      <c r="B94" t="s">
+        <v>71</v>
+      </c>
+      <c r="D94" t="s">
+        <v>72</v>
+      </c>
+      <c r="E94" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A95" s="4">
+        <v>45532.5</v>
+      </c>
+      <c r="B95" t="s">
+        <v>74</v>
+      </c>
+      <c r="D95" t="s">
+        <v>75</v>
+      </c>
+      <c r="E95" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>